<commit_message>
Plantilla: el largo del DNI avisa en vez de bloquear
La base solo exige que el DNI sean dígitos (employees_dni_format_check),
sin largo fijo. La plantilla lo acotaba a 6-9 dígitos con un error que
bloquea la celda, así que un documento legítimo fuera de ese rango dejaba
a esa persona sin poder cargarse.

Queda como advertencia: sugiere el rango y deja seguir. La regla de la
plantilla pasa a ser explícita: bloquea solo donde Postgres también
rechazaría (CUIT y CUIL de 11 dígitos, dotación de 1 a 10, hora de fin
posterior a la de inicio) y avisa donde es una ayuda nuestra.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plantilla-carga-inicial.xlsx
+++ b/docs/plantilla-carga-inicial.xlsx
@@ -19668,10 +19668,10 @@
     <mergeCell ref="A5:O5"/>
   </mergeCells>
   <dataValidations count="12">
-    <dataValidation sqref="A6:A306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="DNI no válido" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222)." type="custom">
+    <dataValidation sqref="A6:A306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revisá el DNI" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222). Si el documento es correcto y tiene otra cantidad de dígitos, aceptá igual." type="custom" errorStyle="warning">
       <formula1>=AND(LEN(A6)&gt;=6,LEN(A6)&lt;=9,ISNUMBER(VALUE(A6)))</formula1>
     </dataValidation>
-    <dataValidation sqref="A4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="DNI no válido" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222)." type="custom">
+    <dataValidation sqref="A4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revisá el DNI" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222). Si el documento es correcto y tiene otra cantidad de dígitos, aceptá igual." type="custom" errorStyle="warning">
       <formula1>=AND(LEN(A4)&gt;=6,LEN(A4)&lt;=9,ISNUMBER(VALUE(A4)))</formula1>
     </dataValidation>
     <dataValidation sqref="E6:E306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tiene que tener 11 dígitos" error="Ingresá los 11 dígitos, sin puntos, guiones ni espacios (por ejemplo 30712345678)." type="custom">
@@ -25029,10 +25029,10 @@
     <mergeCell ref="A5:O5"/>
   </mergeCells>
   <dataValidations count="12">
-    <dataValidation sqref="A6:A306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="DNI no válido" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222)." type="custom">
+    <dataValidation sqref="A6:A306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revisá el DNI" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222). Si el documento es correcto y tiene otra cantidad de dígitos, aceptá igual." type="custom" errorStyle="warning">
       <formula1>=AND(LEN(A6)&gt;=6,LEN(A6)&lt;=9,ISNUMBER(VALUE(A6)))</formula1>
     </dataValidation>
-    <dataValidation sqref="A4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="DNI no válido" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222)." type="custom">
+    <dataValidation sqref="A4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revisá el DNI" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222). Si el documento es correcto y tiene otra cantidad de dígitos, aceptá igual." type="custom" errorStyle="warning">
       <formula1>=AND(LEN(A4)&gt;=6,LEN(A4)&lt;=9,ISNUMBER(VALUE(A4)))</formula1>
     </dataValidation>
     <dataValidation sqref="E6:E306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tiene que tener 11 dígitos" error="Ingresá los 11 dígitos, sin puntos, guiones ni espacios (por ejemplo 30712345678)." type="custom">
@@ -33327,10 +33327,10 @@
     <mergeCell ref="A5:B5"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="A6:A306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="DNI no válido" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222)." type="custom">
+    <dataValidation sqref="A6:A306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revisá el DNI" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222). Si el documento es correcto y tiene otra cantidad de dígitos, aceptá igual." type="custom" errorStyle="warning">
       <formula1>=AND(LEN(A6)&gt;=6,LEN(A6)&lt;=9,ISNUMBER(VALUE(A6)))</formula1>
     </dataValidation>
-    <dataValidation sqref="A4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="DNI no válido" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222)." type="custom">
+    <dataValidation sqref="A4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revisá el DNI" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222). Si el documento es correcto y tiene otra cantidad de dígitos, aceptá igual." type="custom" errorStyle="warning">
       <formula1>=AND(LEN(A4)&gt;=6,LEN(A4)&lt;=9,ISNUMBER(VALUE(A4)))</formula1>
     </dataValidation>
     <dataValidation sqref="B6:B306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Tiene que tener 11 dígitos" error="Ingresá los 11 dígitos, sin puntos, guiones ni espacios (por ejemplo 30712345678)." type="custom">

</xml_diff>

<commit_message>
P24.6: columna de clientes y sedes preferenciales en la planilla y el importador (DATA-001, DATA-003)
- Planilla versión 3: la hoja Supervisores suma «Clientes y sedes preferenciales»
  (lista separada por «;»: «Cliente» para todas sus sedes o «Cliente / Sede»),
  con instrucciones y ejemplo ficticio.
- Importador: valida la columna por fila (cliente o sede inexistente es error con
  hoja, fila y columna; repetidas y redundantes son advertencias) y carga las
  preferencias después de personas y habilitaciones. Respeta --dry-run y --resume;
  la segunda corrida no duplica y «ya existe» (23505) se toma como ya cargado.
- Tests: validación (12 casos) y carga contra una base falsa en memoria (5 casos).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plantilla-carga-inicial.xlsx
+++ b/docs/plantilla-carga-inicial.xlsx
@@ -623,6 +623,11 @@
         <t>Cualquier observación libre.</t>
       </text>
     </comment>
+    <comment ref="P3" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Los clientes y sedes que este coordinador atiende habitualmente: le aparecen primero en su pantalla. No restringe nada: puede tomar cualquier servicio del día. Escribí una lista separada por punto y coma (;). Cada elemento es el cliente (su razón social o su CUIT, vale para todas sus sedes) o "Cliente / Sede" (solo esa sede). Los clientes y sedes tienen que estar en las hojas Clientes y Sedes, escritos igual.</t>
+      </text>
+    </comment>
     <comment ref="A4" authorId="0" shapeId="0">
       <text>
         <t>Esta fila es un EJEMPLO ficticio (ninguna persona ni empresa real). Sirve para que veas cómo se completa cada columna. Borrala antes de devolvernos la planilla.</t>
@@ -1126,7 +1131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B44"/>
+  <dimension ref="B1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1143,7 +1148,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Versión 2 · octubre 2026</t>
+          <t>Versión 3 · octubre 2026</t>
         </is>
       </c>
     </row>
@@ -1196,10 +1201,10 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
+    <row r="11" ht="32" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>•  5. Supervisores — quienes supervisan el trabajo del personal.</t>
+          <t>•  5. Supervisores — los coordinadores: quienes supervisan el trabajo del personal. Ahí también podés indicar los clientes y sedes preferenciales de cada uno.</t>
         </is>
       </c>
     </row>
@@ -1339,54 +1344,110 @@
     <row r="34">
       <c r="B34" s="4" t="inlineStr">
         <is>
+          <t>Sobre los clientes y sedes preferenciales de los coordinadores</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="74" customHeight="1">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>En la hoja Supervisores, la última columna ("Clientes y sedes preferenciales") es opcional. Sirve para que a cada coordinador le aparezcan primero, en su pantalla, los lugares que atiende habitualmente. NO restringe nada: cualquier coordinador puede tomar cualquier servicio del día, y las preferencias solo ordenan la lista. Las coordinadoras y los coordinadores NO se asignan a servicios ni a turnos: eligen ellos cuál supervisar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>•  Escribí una lista separada por punto y coma (;). Cada elemento de la lista es una de estas dos opciones:</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>•  Opción 1 — solo el cliente (su razón social o su CUIT): vale para TODAS sus sedes, también las que se agreguen más adelante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>•  Opción 2 — "Cliente / Sede": el cliente, una barra (/) y el nombre de la sede, igual que en la hoja Sedes. Vale solo para esa sede.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>•  Ejemplo: Ejemplo Limpiezas Del Sur S.A. / Sede Ejemplo Centro; Ejemplo Textiles Norte S.R.L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="46" customHeight="1">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>•  Los clientes y las sedes tienen que estar cargados en las hojas Clientes y Sedes, escritos igual (no importan mayúsculas ni espacios de más). Para un cliente con una sola sede "Principal", alcanza con escribir el cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="46" customHeight="1">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>•  Un coordinador puede tener varias preferencias, y una misma sede puede ser preferida por varios coordinadores. Si algo no coincide, el importador te lo informa con el número de fila, antes de cargar nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
           <t>Sobre las sedes de cada cliente</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="74" customHeight="1">
-      <c r="B35" s="3" t="inlineStr">
+    <row r="44" ht="74" customHeight="1">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Si un cliente tiene un solo domicilio, no hace falta cargarlo en la hoja Sedes: alcanza con la dirección administrativa en la hoja Clientes. Dejá la hoja Sedes sin filas para ese cliente y la plataforma crea sola una sede llamada "Principal" con esa dirección. En la hoja Servicios, para ese cliente, escribí Principal como nombre de la sede. Si el cliente tiene dos o más lugares de trabajo, cargá todos en la hoja Sedes.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="B37" s="4" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Sobre las habilitaciones</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="32" customHeight="1">
-      <c r="B38" s="3" t="inlineStr">
+    <row r="47" ht="32" customHeight="1">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Si una persona no aparece en la hoja Habilitaciones, va a poder trabajar en cualquier cliente. Cargala ahí solamente si querés restringirla a determinados clientes.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" s="4" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Datos personales</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="32" customHeight="1">
-      <c r="B41" s="3" t="inlineStr">
+    <row r="50" ht="32" customHeight="1">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Esta planilla va a tener datos personales reales (DNI, domicilios, teléfonos). Enviánosla por un medio que ustedes consideren seguro y evitá dejarla en carpetas compartidas de acceso público.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="4" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>Ante cualquier duda</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="32" customHeight="1">
-      <c r="B44" s="3" t="inlineStr">
+    <row r="53" ht="32" customHeight="1">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>Escribinos y te ayudamos a completarla. Preferimos una consulta de más a una planilla con datos incompletos o inventados para poder mandarla.</t>
         </is>
@@ -19784,7 +19845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O306"/>
+  <dimension ref="A1:P306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19802,6 +19863,7 @@
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -19814,7 +19876,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Quienes supervisan el trabajo del personal. Si una persona también limpia, cargala además en la hoja Empleados con el mismo DNI.</t>
+          <t>Los coordinadores: quienes supervisan el trabajo del personal. Si una persona también limpia, cargala además en la hoja Empleados con el mismo DNI. No se asignan a servicios: la última columna solo indica sus lugares preferenciales.</t>
         </is>
       </c>
     </row>
@@ -19894,6 +19956,11 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="P3" s="7" t="inlineStr">
+        <is>
+          <t>Clientes y sedes preferenciales</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -19959,6 +20026,11 @@
         </is>
       </c>
       <c r="O4" s="8" t="n"/>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Ejemplo Limpiezas Del Sur S.A. / Sede Ejemplo Centro; Ejemplo Textiles Norte S.R.L.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
@@ -19983,6 +20055,7 @@
       <c r="M6" s="11" t="n"/>
       <c r="N6" s="11" t="n"/>
       <c r="O6" s="11" t="n"/>
+      <c r="P6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="n"/>
@@ -20000,6 +20073,7 @@
       <c r="M7" s="11" t="n"/>
       <c r="N7" s="11" t="n"/>
       <c r="O7" s="11" t="n"/>
+      <c r="P7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n"/>
@@ -20017,6 +20091,7 @@
       <c r="M8" s="11" t="n"/>
       <c r="N8" s="11" t="n"/>
       <c r="O8" s="11" t="n"/>
+      <c r="P8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="n"/>
@@ -20034,6 +20109,7 @@
       <c r="M9" s="11" t="n"/>
       <c r="N9" s="11" t="n"/>
       <c r="O9" s="11" t="n"/>
+      <c r="P9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n"/>
@@ -20051,6 +20127,7 @@
       <c r="M10" s="11" t="n"/>
       <c r="N10" s="11" t="n"/>
       <c r="O10" s="11" t="n"/>
+      <c r="P10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n"/>
@@ -20068,6 +20145,7 @@
       <c r="M11" s="11" t="n"/>
       <c r="N11" s="11" t="n"/>
       <c r="O11" s="11" t="n"/>
+      <c r="P11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n"/>
@@ -20085,6 +20163,7 @@
       <c r="M12" s="11" t="n"/>
       <c r="N12" s="11" t="n"/>
       <c r="O12" s="11" t="n"/>
+      <c r="P12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="n"/>
@@ -20102,6 +20181,7 @@
       <c r="M13" s="11" t="n"/>
       <c r="N13" s="11" t="n"/>
       <c r="O13" s="11" t="n"/>
+      <c r="P13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n"/>
@@ -20119,6 +20199,7 @@
       <c r="M14" s="11" t="n"/>
       <c r="N14" s="11" t="n"/>
       <c r="O14" s="11" t="n"/>
+      <c r="P14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n"/>
@@ -20136,6 +20217,7 @@
       <c r="M15" s="11" t="n"/>
       <c r="N15" s="11" t="n"/>
       <c r="O15" s="11" t="n"/>
+      <c r="P15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
@@ -20153,6 +20235,7 @@
       <c r="M16" s="11" t="n"/>
       <c r="N16" s="11" t="n"/>
       <c r="O16" s="11" t="n"/>
+      <c r="P16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n"/>
@@ -20170,6 +20253,7 @@
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
       <c r="O17" s="11" t="n"/>
+      <c r="P17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -20187,6 +20271,7 @@
       <c r="M18" s="11" t="n"/>
       <c r="N18" s="11" t="n"/>
       <c r="O18" s="11" t="n"/>
+      <c r="P18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n"/>
@@ -20204,6 +20289,7 @@
       <c r="M19" s="11" t="n"/>
       <c r="N19" s="11" t="n"/>
       <c r="O19" s="11" t="n"/>
+      <c r="P19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -20221,6 +20307,7 @@
       <c r="M20" s="11" t="n"/>
       <c r="N20" s="11" t="n"/>
       <c r="O20" s="11" t="n"/>
+      <c r="P20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n"/>
@@ -20238,6 +20325,7 @@
       <c r="M21" s="11" t="n"/>
       <c r="N21" s="11" t="n"/>
       <c r="O21" s="11" t="n"/>
+      <c r="P21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -20255,6 +20343,7 @@
       <c r="M22" s="11" t="n"/>
       <c r="N22" s="11" t="n"/>
       <c r="O22" s="11" t="n"/>
+      <c r="P22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n"/>
@@ -20272,6 +20361,7 @@
       <c r="M23" s="11" t="n"/>
       <c r="N23" s="11" t="n"/>
       <c r="O23" s="11" t="n"/>
+      <c r="P23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -20289,6 +20379,7 @@
       <c r="M24" s="11" t="n"/>
       <c r="N24" s="11" t="n"/>
       <c r="O24" s="11" t="n"/>
+      <c r="P24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n"/>
@@ -20306,6 +20397,7 @@
       <c r="M25" s="11" t="n"/>
       <c r="N25" s="11" t="n"/>
       <c r="O25" s="11" t="n"/>
+      <c r="P25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -20323,6 +20415,7 @@
       <c r="M26" s="11" t="n"/>
       <c r="N26" s="11" t="n"/>
       <c r="O26" s="11" t="n"/>
+      <c r="P26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n"/>
@@ -20340,6 +20433,7 @@
       <c r="M27" s="11" t="n"/>
       <c r="N27" s="11" t="n"/>
       <c r="O27" s="11" t="n"/>
+      <c r="P27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -20357,6 +20451,7 @@
       <c r="M28" s="11" t="n"/>
       <c r="N28" s="11" t="n"/>
       <c r="O28" s="11" t="n"/>
+      <c r="P28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n"/>
@@ -20374,6 +20469,7 @@
       <c r="M29" s="11" t="n"/>
       <c r="N29" s="11" t="n"/>
       <c r="O29" s="11" t="n"/>
+      <c r="P29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -20391,6 +20487,7 @@
       <c r="M30" s="11" t="n"/>
       <c r="N30" s="11" t="n"/>
       <c r="O30" s="11" t="n"/>
+      <c r="P30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n"/>
@@ -20408,6 +20505,7 @@
       <c r="M31" s="11" t="n"/>
       <c r="N31" s="11" t="n"/>
       <c r="O31" s="11" t="n"/>
+      <c r="P31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -20425,6 +20523,7 @@
       <c r="M32" s="11" t="n"/>
       <c r="N32" s="11" t="n"/>
       <c r="O32" s="11" t="n"/>
+      <c r="P32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n"/>
@@ -20442,6 +20541,7 @@
       <c r="M33" s="11" t="n"/>
       <c r="N33" s="11" t="n"/>
       <c r="O33" s="11" t="n"/>
+      <c r="P33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -20459,6 +20559,7 @@
       <c r="M34" s="11" t="n"/>
       <c r="N34" s="11" t="n"/>
       <c r="O34" s="11" t="n"/>
+      <c r="P34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="n"/>
@@ -20476,6 +20577,7 @@
       <c r="M35" s="11" t="n"/>
       <c r="N35" s="11" t="n"/>
       <c r="O35" s="11" t="n"/>
+      <c r="P35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -20493,6 +20595,7 @@
       <c r="M36" s="11" t="n"/>
       <c r="N36" s="11" t="n"/>
       <c r="O36" s="11" t="n"/>
+      <c r="P36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n"/>
@@ -20510,6 +20613,7 @@
       <c r="M37" s="11" t="n"/>
       <c r="N37" s="11" t="n"/>
       <c r="O37" s="11" t="n"/>
+      <c r="P37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -20527,6 +20631,7 @@
       <c r="M38" s="11" t="n"/>
       <c r="N38" s="11" t="n"/>
       <c r="O38" s="11" t="n"/>
+      <c r="P38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n"/>
@@ -20544,6 +20649,7 @@
       <c r="M39" s="11" t="n"/>
       <c r="N39" s="11" t="n"/>
       <c r="O39" s="11" t="n"/>
+      <c r="P39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n"/>
@@ -20561,6 +20667,7 @@
       <c r="M40" s="11" t="n"/>
       <c r="N40" s="11" t="n"/>
       <c r="O40" s="11" t="n"/>
+      <c r="P40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n"/>
@@ -20578,6 +20685,7 @@
       <c r="M41" s="11" t="n"/>
       <c r="N41" s="11" t="n"/>
       <c r="O41" s="11" t="n"/>
+      <c r="P41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n"/>
@@ -20595,6 +20703,7 @@
       <c r="M42" s="11" t="n"/>
       <c r="N42" s="11" t="n"/>
       <c r="O42" s="11" t="n"/>
+      <c r="P42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n"/>
@@ -20612,6 +20721,7 @@
       <c r="M43" s="11" t="n"/>
       <c r="N43" s="11" t="n"/>
       <c r="O43" s="11" t="n"/>
+      <c r="P43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n"/>
@@ -20629,6 +20739,7 @@
       <c r="M44" s="11" t="n"/>
       <c r="N44" s="11" t="n"/>
       <c r="O44" s="11" t="n"/>
+      <c r="P44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n"/>
@@ -20646,6 +20757,7 @@
       <c r="M45" s="11" t="n"/>
       <c r="N45" s="11" t="n"/>
       <c r="O45" s="11" t="n"/>
+      <c r="P45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
@@ -20663,6 +20775,7 @@
       <c r="M46" s="11" t="n"/>
       <c r="N46" s="11" t="n"/>
       <c r="O46" s="11" t="n"/>
+      <c r="P46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="n"/>
@@ -20680,6 +20793,7 @@
       <c r="M47" s="11" t="n"/>
       <c r="N47" s="11" t="n"/>
       <c r="O47" s="11" t="n"/>
+      <c r="P47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n"/>
@@ -20697,6 +20811,7 @@
       <c r="M48" s="11" t="n"/>
       <c r="N48" s="11" t="n"/>
       <c r="O48" s="11" t="n"/>
+      <c r="P48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="n"/>
@@ -20714,6 +20829,7 @@
       <c r="M49" s="11" t="n"/>
       <c r="N49" s="11" t="n"/>
       <c r="O49" s="11" t="n"/>
+      <c r="P49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n"/>
@@ -20731,6 +20847,7 @@
       <c r="M50" s="11" t="n"/>
       <c r="N50" s="11" t="n"/>
       <c r="O50" s="11" t="n"/>
+      <c r="P50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="n"/>
@@ -20748,6 +20865,7 @@
       <c r="M51" s="11" t="n"/>
       <c r="N51" s="11" t="n"/>
       <c r="O51" s="11" t="n"/>
+      <c r="P51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n"/>
@@ -20765,6 +20883,7 @@
       <c r="M52" s="11" t="n"/>
       <c r="N52" s="11" t="n"/>
       <c r="O52" s="11" t="n"/>
+      <c r="P52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n"/>
@@ -20782,6 +20901,7 @@
       <c r="M53" s="11" t="n"/>
       <c r="N53" s="11" t="n"/>
       <c r="O53" s="11" t="n"/>
+      <c r="P53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n"/>
@@ -20799,6 +20919,7 @@
       <c r="M54" s="11" t="n"/>
       <c r="N54" s="11" t="n"/>
       <c r="O54" s="11" t="n"/>
+      <c r="P54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="n"/>
@@ -20816,6 +20937,7 @@
       <c r="M55" s="11" t="n"/>
       <c r="N55" s="11" t="n"/>
       <c r="O55" s="11" t="n"/>
+      <c r="P55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n"/>
@@ -20833,6 +20955,7 @@
       <c r="M56" s="11" t="n"/>
       <c r="N56" s="11" t="n"/>
       <c r="O56" s="11" t="n"/>
+      <c r="P56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="n"/>
@@ -20850,6 +20973,7 @@
       <c r="M57" s="11" t="n"/>
       <c r="N57" s="11" t="n"/>
       <c r="O57" s="11" t="n"/>
+      <c r="P57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n"/>
@@ -20867,6 +20991,7 @@
       <c r="M58" s="11" t="n"/>
       <c r="N58" s="11" t="n"/>
       <c r="O58" s="11" t="n"/>
+      <c r="P58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="n"/>
@@ -20884,6 +21009,7 @@
       <c r="M59" s="11" t="n"/>
       <c r="N59" s="11" t="n"/>
       <c r="O59" s="11" t="n"/>
+      <c r="P59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n"/>
@@ -20901,6 +21027,7 @@
       <c r="M60" s="11" t="n"/>
       <c r="N60" s="11" t="n"/>
       <c r="O60" s="11" t="n"/>
+      <c r="P60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
@@ -20918,6 +21045,7 @@
       <c r="M61" s="11" t="n"/>
       <c r="N61" s="11" t="n"/>
       <c r="O61" s="11" t="n"/>
+      <c r="P61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n"/>
@@ -20935,6 +21063,7 @@
       <c r="M62" s="11" t="n"/>
       <c r="N62" s="11" t="n"/>
       <c r="O62" s="11" t="n"/>
+      <c r="P62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="n"/>
@@ -20952,6 +21081,7 @@
       <c r="M63" s="11" t="n"/>
       <c r="N63" s="11" t="n"/>
       <c r="O63" s="11" t="n"/>
+      <c r="P63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="n"/>
@@ -20969,6 +21099,7 @@
       <c r="M64" s="11" t="n"/>
       <c r="N64" s="11" t="n"/>
       <c r="O64" s="11" t="n"/>
+      <c r="P64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="10" t="n"/>
@@ -20986,6 +21117,7 @@
       <c r="M65" s="11" t="n"/>
       <c r="N65" s="11" t="n"/>
       <c r="O65" s="11" t="n"/>
+      <c r="P65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="n"/>
@@ -21003,6 +21135,7 @@
       <c r="M66" s="11" t="n"/>
       <c r="N66" s="11" t="n"/>
       <c r="O66" s="11" t="n"/>
+      <c r="P66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="10" t="n"/>
@@ -21020,6 +21153,7 @@
       <c r="M67" s="11" t="n"/>
       <c r="N67" s="11" t="n"/>
       <c r="O67" s="11" t="n"/>
+      <c r="P67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n"/>
@@ -21037,6 +21171,7 @@
       <c r="M68" s="11" t="n"/>
       <c r="N68" s="11" t="n"/>
       <c r="O68" s="11" t="n"/>
+      <c r="P68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="10" t="n"/>
@@ -21054,6 +21189,7 @@
       <c r="M69" s="11" t="n"/>
       <c r="N69" s="11" t="n"/>
       <c r="O69" s="11" t="n"/>
+      <c r="P69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="n"/>
@@ -21071,6 +21207,7 @@
       <c r="M70" s="11" t="n"/>
       <c r="N70" s="11" t="n"/>
       <c r="O70" s="11" t="n"/>
+      <c r="P70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="10" t="n"/>
@@ -21088,6 +21225,7 @@
       <c r="M71" s="11" t="n"/>
       <c r="N71" s="11" t="n"/>
       <c r="O71" s="11" t="n"/>
+      <c r="P71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="n"/>
@@ -21105,6 +21243,7 @@
       <c r="M72" s="11" t="n"/>
       <c r="N72" s="11" t="n"/>
       <c r="O72" s="11" t="n"/>
+      <c r="P72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="n"/>
@@ -21122,6 +21261,7 @@
       <c r="M73" s="11" t="n"/>
       <c r="N73" s="11" t="n"/>
       <c r="O73" s="11" t="n"/>
+      <c r="P73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="n"/>
@@ -21139,6 +21279,7 @@
       <c r="M74" s="11" t="n"/>
       <c r="N74" s="11" t="n"/>
       <c r="O74" s="11" t="n"/>
+      <c r="P74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="10" t="n"/>
@@ -21156,6 +21297,7 @@
       <c r="M75" s="11" t="n"/>
       <c r="N75" s="11" t="n"/>
       <c r="O75" s="11" t="n"/>
+      <c r="P75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n"/>
@@ -21173,6 +21315,7 @@
       <c r="M76" s="11" t="n"/>
       <c r="N76" s="11" t="n"/>
       <c r="O76" s="11" t="n"/>
+      <c r="P76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="n"/>
@@ -21190,6 +21333,7 @@
       <c r="M77" s="11" t="n"/>
       <c r="N77" s="11" t="n"/>
       <c r="O77" s="11" t="n"/>
+      <c r="P77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="n"/>
@@ -21207,6 +21351,7 @@
       <c r="M78" s="11" t="n"/>
       <c r="N78" s="11" t="n"/>
       <c r="O78" s="11" t="n"/>
+      <c r="P78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="10" t="n"/>
@@ -21224,6 +21369,7 @@
       <c r="M79" s="11" t="n"/>
       <c r="N79" s="11" t="n"/>
       <c r="O79" s="11" t="n"/>
+      <c r="P79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="n"/>
@@ -21241,6 +21387,7 @@
       <c r="M80" s="11" t="n"/>
       <c r="N80" s="11" t="n"/>
       <c r="O80" s="11" t="n"/>
+      <c r="P80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="n"/>
@@ -21258,6 +21405,7 @@
       <c r="M81" s="11" t="n"/>
       <c r="N81" s="11" t="n"/>
       <c r="O81" s="11" t="n"/>
+      <c r="P81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="n"/>
@@ -21275,6 +21423,7 @@
       <c r="M82" s="11" t="n"/>
       <c r="N82" s="11" t="n"/>
       <c r="O82" s="11" t="n"/>
+      <c r="P82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="10" t="n"/>
@@ -21292,6 +21441,7 @@
       <c r="M83" s="11" t="n"/>
       <c r="N83" s="11" t="n"/>
       <c r="O83" s="11" t="n"/>
+      <c r="P83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="n"/>
@@ -21309,6 +21459,7 @@
       <c r="M84" s="11" t="n"/>
       <c r="N84" s="11" t="n"/>
       <c r="O84" s="11" t="n"/>
+      <c r="P84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="n"/>
@@ -21326,6 +21477,7 @@
       <c r="M85" s="11" t="n"/>
       <c r="N85" s="11" t="n"/>
       <c r="O85" s="11" t="n"/>
+      <c r="P85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="n"/>
@@ -21343,6 +21495,7 @@
       <c r="M86" s="11" t="n"/>
       <c r="N86" s="11" t="n"/>
       <c r="O86" s="11" t="n"/>
+      <c r="P86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="n"/>
@@ -21360,6 +21513,7 @@
       <c r="M87" s="11" t="n"/>
       <c r="N87" s="11" t="n"/>
       <c r="O87" s="11" t="n"/>
+      <c r="P87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="n"/>
@@ -21377,6 +21531,7 @@
       <c r="M88" s="11" t="n"/>
       <c r="N88" s="11" t="n"/>
       <c r="O88" s="11" t="n"/>
+      <c r="P88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="10" t="n"/>
@@ -21394,6 +21549,7 @@
       <c r="M89" s="11" t="n"/>
       <c r="N89" s="11" t="n"/>
       <c r="O89" s="11" t="n"/>
+      <c r="P89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="n"/>
@@ -21411,6 +21567,7 @@
       <c r="M90" s="11" t="n"/>
       <c r="N90" s="11" t="n"/>
       <c r="O90" s="11" t="n"/>
+      <c r="P90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="n"/>
@@ -21428,6 +21585,7 @@
       <c r="M91" s="11" t="n"/>
       <c r="N91" s="11" t="n"/>
       <c r="O91" s="11" t="n"/>
+      <c r="P91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n"/>
@@ -21445,6 +21603,7 @@
       <c r="M92" s="11" t="n"/>
       <c r="N92" s="11" t="n"/>
       <c r="O92" s="11" t="n"/>
+      <c r="P92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="n"/>
@@ -21462,6 +21621,7 @@
       <c r="M93" s="11" t="n"/>
       <c r="N93" s="11" t="n"/>
       <c r="O93" s="11" t="n"/>
+      <c r="P93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n"/>
@@ -21479,6 +21639,7 @@
       <c r="M94" s="11" t="n"/>
       <c r="N94" s="11" t="n"/>
       <c r="O94" s="11" t="n"/>
+      <c r="P94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="n"/>
@@ -21496,6 +21657,7 @@
       <c r="M95" s="11" t="n"/>
       <c r="N95" s="11" t="n"/>
       <c r="O95" s="11" t="n"/>
+      <c r="P95" s="11" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="n"/>
@@ -21513,6 +21675,7 @@
       <c r="M96" s="11" t="n"/>
       <c r="N96" s="11" t="n"/>
       <c r="O96" s="11" t="n"/>
+      <c r="P96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="10" t="n"/>
@@ -21530,6 +21693,7 @@
       <c r="M97" s="11" t="n"/>
       <c r="N97" s="11" t="n"/>
       <c r="O97" s="11" t="n"/>
+      <c r="P97" s="11" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="n"/>
@@ -21547,6 +21711,7 @@
       <c r="M98" s="11" t="n"/>
       <c r="N98" s="11" t="n"/>
       <c r="O98" s="11" t="n"/>
+      <c r="P98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="10" t="n"/>
@@ -21564,6 +21729,7 @@
       <c r="M99" s="11" t="n"/>
       <c r="N99" s="11" t="n"/>
       <c r="O99" s="11" t="n"/>
+      <c r="P99" s="11" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="n"/>
@@ -21581,6 +21747,7 @@
       <c r="M100" s="11" t="n"/>
       <c r="N100" s="11" t="n"/>
       <c r="O100" s="11" t="n"/>
+      <c r="P100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="n"/>
@@ -21598,6 +21765,7 @@
       <c r="M101" s="11" t="n"/>
       <c r="N101" s="11" t="n"/>
       <c r="O101" s="11" t="n"/>
+      <c r="P101" s="11" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="n"/>
@@ -21615,6 +21783,7 @@
       <c r="M102" s="11" t="n"/>
       <c r="N102" s="11" t="n"/>
       <c r="O102" s="11" t="n"/>
+      <c r="P102" s="11" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="10" t="n"/>
@@ -21632,6 +21801,7 @@
       <c r="M103" s="11" t="n"/>
       <c r="N103" s="11" t="n"/>
       <c r="O103" s="11" t="n"/>
+      <c r="P103" s="11" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="n"/>
@@ -21649,6 +21819,7 @@
       <c r="M104" s="11" t="n"/>
       <c r="N104" s="11" t="n"/>
       <c r="O104" s="11" t="n"/>
+      <c r="P104" s="11" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="10" t="n"/>
@@ -21666,6 +21837,7 @@
       <c r="M105" s="11" t="n"/>
       <c r="N105" s="11" t="n"/>
       <c r="O105" s="11" t="n"/>
+      <c r="P105" s="11" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="n"/>
@@ -21683,6 +21855,7 @@
       <c r="M106" s="11" t="n"/>
       <c r="N106" s="11" t="n"/>
       <c r="O106" s="11" t="n"/>
+      <c r="P106" s="11" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="10" t="n"/>
@@ -21700,6 +21873,7 @@
       <c r="M107" s="11" t="n"/>
       <c r="N107" s="11" t="n"/>
       <c r="O107" s="11" t="n"/>
+      <c r="P107" s="11" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="10" t="n"/>
@@ -21717,6 +21891,7 @@
       <c r="M108" s="11" t="n"/>
       <c r="N108" s="11" t="n"/>
       <c r="O108" s="11" t="n"/>
+      <c r="P108" s="11" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="10" t="n"/>
@@ -21734,6 +21909,7 @@
       <c r="M109" s="11" t="n"/>
       <c r="N109" s="11" t="n"/>
       <c r="O109" s="11" t="n"/>
+      <c r="P109" s="11" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="n"/>
@@ -21751,6 +21927,7 @@
       <c r="M110" s="11" t="n"/>
       <c r="N110" s="11" t="n"/>
       <c r="O110" s="11" t="n"/>
+      <c r="P110" s="11" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="10" t="n"/>
@@ -21768,6 +21945,7 @@
       <c r="M111" s="11" t="n"/>
       <c r="N111" s="11" t="n"/>
       <c r="O111" s="11" t="n"/>
+      <c r="P111" s="11" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="10" t="n"/>
@@ -21785,6 +21963,7 @@
       <c r="M112" s="11" t="n"/>
       <c r="N112" s="11" t="n"/>
       <c r="O112" s="11" t="n"/>
+      <c r="P112" s="11" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="10" t="n"/>
@@ -21802,6 +21981,7 @@
       <c r="M113" s="11" t="n"/>
       <c r="N113" s="11" t="n"/>
       <c r="O113" s="11" t="n"/>
+      <c r="P113" s="11" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="10" t="n"/>
@@ -21819,6 +21999,7 @@
       <c r="M114" s="11" t="n"/>
       <c r="N114" s="11" t="n"/>
       <c r="O114" s="11" t="n"/>
+      <c r="P114" s="11" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="10" t="n"/>
@@ -21836,6 +22017,7 @@
       <c r="M115" s="11" t="n"/>
       <c r="N115" s="11" t="n"/>
       <c r="O115" s="11" t="n"/>
+      <c r="P115" s="11" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="10" t="n"/>
@@ -21853,6 +22035,7 @@
       <c r="M116" s="11" t="n"/>
       <c r="N116" s="11" t="n"/>
       <c r="O116" s="11" t="n"/>
+      <c r="P116" s="11" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="10" t="n"/>
@@ -21870,6 +22053,7 @@
       <c r="M117" s="11" t="n"/>
       <c r="N117" s="11" t="n"/>
       <c r="O117" s="11" t="n"/>
+      <c r="P117" s="11" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="10" t="n"/>
@@ -21887,6 +22071,7 @@
       <c r="M118" s="11" t="n"/>
       <c r="N118" s="11" t="n"/>
       <c r="O118" s="11" t="n"/>
+      <c r="P118" s="11" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="10" t="n"/>
@@ -21904,6 +22089,7 @@
       <c r="M119" s="11" t="n"/>
       <c r="N119" s="11" t="n"/>
       <c r="O119" s="11" t="n"/>
+      <c r="P119" s="11" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="10" t="n"/>
@@ -21921,6 +22107,7 @@
       <c r="M120" s="11" t="n"/>
       <c r="N120" s="11" t="n"/>
       <c r="O120" s="11" t="n"/>
+      <c r="P120" s="11" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="10" t="n"/>
@@ -21938,6 +22125,7 @@
       <c r="M121" s="11" t="n"/>
       <c r="N121" s="11" t="n"/>
       <c r="O121" s="11" t="n"/>
+      <c r="P121" s="11" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="10" t="n"/>
@@ -21955,6 +22143,7 @@
       <c r="M122" s="11" t="n"/>
       <c r="N122" s="11" t="n"/>
       <c r="O122" s="11" t="n"/>
+      <c r="P122" s="11" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="10" t="n"/>
@@ -21972,6 +22161,7 @@
       <c r="M123" s="11" t="n"/>
       <c r="N123" s="11" t="n"/>
       <c r="O123" s="11" t="n"/>
+      <c r="P123" s="11" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="10" t="n"/>
@@ -21989,6 +22179,7 @@
       <c r="M124" s="11" t="n"/>
       <c r="N124" s="11" t="n"/>
       <c r="O124" s="11" t="n"/>
+      <c r="P124" s="11" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="10" t="n"/>
@@ -22006,6 +22197,7 @@
       <c r="M125" s="11" t="n"/>
       <c r="N125" s="11" t="n"/>
       <c r="O125" s="11" t="n"/>
+      <c r="P125" s="11" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="10" t="n"/>
@@ -22023,6 +22215,7 @@
       <c r="M126" s="11" t="n"/>
       <c r="N126" s="11" t="n"/>
       <c r="O126" s="11" t="n"/>
+      <c r="P126" s="11" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="10" t="n"/>
@@ -22040,6 +22233,7 @@
       <c r="M127" s="11" t="n"/>
       <c r="N127" s="11" t="n"/>
       <c r="O127" s="11" t="n"/>
+      <c r="P127" s="11" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="10" t="n"/>
@@ -22057,6 +22251,7 @@
       <c r="M128" s="11" t="n"/>
       <c r="N128" s="11" t="n"/>
       <c r="O128" s="11" t="n"/>
+      <c r="P128" s="11" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="10" t="n"/>
@@ -22074,6 +22269,7 @@
       <c r="M129" s="11" t="n"/>
       <c r="N129" s="11" t="n"/>
       <c r="O129" s="11" t="n"/>
+      <c r="P129" s="11" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="10" t="n"/>
@@ -22091,6 +22287,7 @@
       <c r="M130" s="11" t="n"/>
       <c r="N130" s="11" t="n"/>
       <c r="O130" s="11" t="n"/>
+      <c r="P130" s="11" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="10" t="n"/>
@@ -22108,6 +22305,7 @@
       <c r="M131" s="11" t="n"/>
       <c r="N131" s="11" t="n"/>
       <c r="O131" s="11" t="n"/>
+      <c r="P131" s="11" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="10" t="n"/>
@@ -22125,6 +22323,7 @@
       <c r="M132" s="11" t="n"/>
       <c r="N132" s="11" t="n"/>
       <c r="O132" s="11" t="n"/>
+      <c r="P132" s="11" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="10" t="n"/>
@@ -22142,6 +22341,7 @@
       <c r="M133" s="11" t="n"/>
       <c r="N133" s="11" t="n"/>
       <c r="O133" s="11" t="n"/>
+      <c r="P133" s="11" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="10" t="n"/>
@@ -22159,6 +22359,7 @@
       <c r="M134" s="11" t="n"/>
       <c r="N134" s="11" t="n"/>
       <c r="O134" s="11" t="n"/>
+      <c r="P134" s="11" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="10" t="n"/>
@@ -22176,6 +22377,7 @@
       <c r="M135" s="11" t="n"/>
       <c r="N135" s="11" t="n"/>
       <c r="O135" s="11" t="n"/>
+      <c r="P135" s="11" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="10" t="n"/>
@@ -22193,6 +22395,7 @@
       <c r="M136" s="11" t="n"/>
       <c r="N136" s="11" t="n"/>
       <c r="O136" s="11" t="n"/>
+      <c r="P136" s="11" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="10" t="n"/>
@@ -22210,6 +22413,7 @@
       <c r="M137" s="11" t="n"/>
       <c r="N137" s="11" t="n"/>
       <c r="O137" s="11" t="n"/>
+      <c r="P137" s="11" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="10" t="n"/>
@@ -22227,6 +22431,7 @@
       <c r="M138" s="11" t="n"/>
       <c r="N138" s="11" t="n"/>
       <c r="O138" s="11" t="n"/>
+      <c r="P138" s="11" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="10" t="n"/>
@@ -22244,6 +22449,7 @@
       <c r="M139" s="11" t="n"/>
       <c r="N139" s="11" t="n"/>
       <c r="O139" s="11" t="n"/>
+      <c r="P139" s="11" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="10" t="n"/>
@@ -22261,6 +22467,7 @@
       <c r="M140" s="11" t="n"/>
       <c r="N140" s="11" t="n"/>
       <c r="O140" s="11" t="n"/>
+      <c r="P140" s="11" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="10" t="n"/>
@@ -22278,6 +22485,7 @@
       <c r="M141" s="11" t="n"/>
       <c r="N141" s="11" t="n"/>
       <c r="O141" s="11" t="n"/>
+      <c r="P141" s="11" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="10" t="n"/>
@@ -22295,6 +22503,7 @@
       <c r="M142" s="11" t="n"/>
       <c r="N142" s="11" t="n"/>
       <c r="O142" s="11" t="n"/>
+      <c r="P142" s="11" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="10" t="n"/>
@@ -22312,6 +22521,7 @@
       <c r="M143" s="11" t="n"/>
       <c r="N143" s="11" t="n"/>
       <c r="O143" s="11" t="n"/>
+      <c r="P143" s="11" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="10" t="n"/>
@@ -22329,6 +22539,7 @@
       <c r="M144" s="11" t="n"/>
       <c r="N144" s="11" t="n"/>
       <c r="O144" s="11" t="n"/>
+      <c r="P144" s="11" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="10" t="n"/>
@@ -22346,6 +22557,7 @@
       <c r="M145" s="11" t="n"/>
       <c r="N145" s="11" t="n"/>
       <c r="O145" s="11" t="n"/>
+      <c r="P145" s="11" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="10" t="n"/>
@@ -22363,6 +22575,7 @@
       <c r="M146" s="11" t="n"/>
       <c r="N146" s="11" t="n"/>
       <c r="O146" s="11" t="n"/>
+      <c r="P146" s="11" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="10" t="n"/>
@@ -22380,6 +22593,7 @@
       <c r="M147" s="11" t="n"/>
       <c r="N147" s="11" t="n"/>
       <c r="O147" s="11" t="n"/>
+      <c r="P147" s="11" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="10" t="n"/>
@@ -22397,6 +22611,7 @@
       <c r="M148" s="11" t="n"/>
       <c r="N148" s="11" t="n"/>
       <c r="O148" s="11" t="n"/>
+      <c r="P148" s="11" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="10" t="n"/>
@@ -22414,6 +22629,7 @@
       <c r="M149" s="11" t="n"/>
       <c r="N149" s="11" t="n"/>
       <c r="O149" s="11" t="n"/>
+      <c r="P149" s="11" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="10" t="n"/>
@@ -22431,6 +22647,7 @@
       <c r="M150" s="11" t="n"/>
       <c r="N150" s="11" t="n"/>
       <c r="O150" s="11" t="n"/>
+      <c r="P150" s="11" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="10" t="n"/>
@@ -22448,6 +22665,7 @@
       <c r="M151" s="11" t="n"/>
       <c r="N151" s="11" t="n"/>
       <c r="O151" s="11" t="n"/>
+      <c r="P151" s="11" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="10" t="n"/>
@@ -22465,6 +22683,7 @@
       <c r="M152" s="11" t="n"/>
       <c r="N152" s="11" t="n"/>
       <c r="O152" s="11" t="n"/>
+      <c r="P152" s="11" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="10" t="n"/>
@@ -22482,6 +22701,7 @@
       <c r="M153" s="11" t="n"/>
       <c r="N153" s="11" t="n"/>
       <c r="O153" s="11" t="n"/>
+      <c r="P153" s="11" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="10" t="n"/>
@@ -22499,6 +22719,7 @@
       <c r="M154" s="11" t="n"/>
       <c r="N154" s="11" t="n"/>
       <c r="O154" s="11" t="n"/>
+      <c r="P154" s="11" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="10" t="n"/>
@@ -22516,6 +22737,7 @@
       <c r="M155" s="11" t="n"/>
       <c r="N155" s="11" t="n"/>
       <c r="O155" s="11" t="n"/>
+      <c r="P155" s="11" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="10" t="n"/>
@@ -22533,6 +22755,7 @@
       <c r="M156" s="11" t="n"/>
       <c r="N156" s="11" t="n"/>
       <c r="O156" s="11" t="n"/>
+      <c r="P156" s="11" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="10" t="n"/>
@@ -22550,6 +22773,7 @@
       <c r="M157" s="11" t="n"/>
       <c r="N157" s="11" t="n"/>
       <c r="O157" s="11" t="n"/>
+      <c r="P157" s="11" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="10" t="n"/>
@@ -22567,6 +22791,7 @@
       <c r="M158" s="11" t="n"/>
       <c r="N158" s="11" t="n"/>
       <c r="O158" s="11" t="n"/>
+      <c r="P158" s="11" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="10" t="n"/>
@@ -22584,6 +22809,7 @@
       <c r="M159" s="11" t="n"/>
       <c r="N159" s="11" t="n"/>
       <c r="O159" s="11" t="n"/>
+      <c r="P159" s="11" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="10" t="n"/>
@@ -22601,6 +22827,7 @@
       <c r="M160" s="11" t="n"/>
       <c r="N160" s="11" t="n"/>
       <c r="O160" s="11" t="n"/>
+      <c r="P160" s="11" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="10" t="n"/>
@@ -22618,6 +22845,7 @@
       <c r="M161" s="11" t="n"/>
       <c r="N161" s="11" t="n"/>
       <c r="O161" s="11" t="n"/>
+      <c r="P161" s="11" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="10" t="n"/>
@@ -22635,6 +22863,7 @@
       <c r="M162" s="11" t="n"/>
       <c r="N162" s="11" t="n"/>
       <c r="O162" s="11" t="n"/>
+      <c r="P162" s="11" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="10" t="n"/>
@@ -22652,6 +22881,7 @@
       <c r="M163" s="11" t="n"/>
       <c r="N163" s="11" t="n"/>
       <c r="O163" s="11" t="n"/>
+      <c r="P163" s="11" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="10" t="n"/>
@@ -22669,6 +22899,7 @@
       <c r="M164" s="11" t="n"/>
       <c r="N164" s="11" t="n"/>
       <c r="O164" s="11" t="n"/>
+      <c r="P164" s="11" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="10" t="n"/>
@@ -22686,6 +22917,7 @@
       <c r="M165" s="11" t="n"/>
       <c r="N165" s="11" t="n"/>
       <c r="O165" s="11" t="n"/>
+      <c r="P165" s="11" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="10" t="n"/>
@@ -22703,6 +22935,7 @@
       <c r="M166" s="11" t="n"/>
       <c r="N166" s="11" t="n"/>
       <c r="O166" s="11" t="n"/>
+      <c r="P166" s="11" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="10" t="n"/>
@@ -22720,6 +22953,7 @@
       <c r="M167" s="11" t="n"/>
       <c r="N167" s="11" t="n"/>
       <c r="O167" s="11" t="n"/>
+      <c r="P167" s="11" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="10" t="n"/>
@@ -22737,6 +22971,7 @@
       <c r="M168" s="11" t="n"/>
       <c r="N168" s="11" t="n"/>
       <c r="O168" s="11" t="n"/>
+      <c r="P168" s="11" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="10" t="n"/>
@@ -22754,6 +22989,7 @@
       <c r="M169" s="11" t="n"/>
       <c r="N169" s="11" t="n"/>
       <c r="O169" s="11" t="n"/>
+      <c r="P169" s="11" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="10" t="n"/>
@@ -22771,6 +23007,7 @@
       <c r="M170" s="11" t="n"/>
       <c r="N170" s="11" t="n"/>
       <c r="O170" s="11" t="n"/>
+      <c r="P170" s="11" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="10" t="n"/>
@@ -22788,6 +23025,7 @@
       <c r="M171" s="11" t="n"/>
       <c r="N171" s="11" t="n"/>
       <c r="O171" s="11" t="n"/>
+      <c r="P171" s="11" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="10" t="n"/>
@@ -22805,6 +23043,7 @@
       <c r="M172" s="11" t="n"/>
       <c r="N172" s="11" t="n"/>
       <c r="O172" s="11" t="n"/>
+      <c r="P172" s="11" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="10" t="n"/>
@@ -22822,6 +23061,7 @@
       <c r="M173" s="11" t="n"/>
       <c r="N173" s="11" t="n"/>
       <c r="O173" s="11" t="n"/>
+      <c r="P173" s="11" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="10" t="n"/>
@@ -22839,6 +23079,7 @@
       <c r="M174" s="11" t="n"/>
       <c r="N174" s="11" t="n"/>
       <c r="O174" s="11" t="n"/>
+      <c r="P174" s="11" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="10" t="n"/>
@@ -22856,6 +23097,7 @@
       <c r="M175" s="11" t="n"/>
       <c r="N175" s="11" t="n"/>
       <c r="O175" s="11" t="n"/>
+      <c r="P175" s="11" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="10" t="n"/>
@@ -22873,6 +23115,7 @@
       <c r="M176" s="11" t="n"/>
       <c r="N176" s="11" t="n"/>
       <c r="O176" s="11" t="n"/>
+      <c r="P176" s="11" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="10" t="n"/>
@@ -22890,6 +23133,7 @@
       <c r="M177" s="11" t="n"/>
       <c r="N177" s="11" t="n"/>
       <c r="O177" s="11" t="n"/>
+      <c r="P177" s="11" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="10" t="n"/>
@@ -22907,6 +23151,7 @@
       <c r="M178" s="11" t="n"/>
       <c r="N178" s="11" t="n"/>
       <c r="O178" s="11" t="n"/>
+      <c r="P178" s="11" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="10" t="n"/>
@@ -22924,6 +23169,7 @@
       <c r="M179" s="11" t="n"/>
       <c r="N179" s="11" t="n"/>
       <c r="O179" s="11" t="n"/>
+      <c r="P179" s="11" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="10" t="n"/>
@@ -22941,6 +23187,7 @@
       <c r="M180" s="11" t="n"/>
       <c r="N180" s="11" t="n"/>
       <c r="O180" s="11" t="n"/>
+      <c r="P180" s="11" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="10" t="n"/>
@@ -22958,6 +23205,7 @@
       <c r="M181" s="11" t="n"/>
       <c r="N181" s="11" t="n"/>
       <c r="O181" s="11" t="n"/>
+      <c r="P181" s="11" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="10" t="n"/>
@@ -22975,6 +23223,7 @@
       <c r="M182" s="11" t="n"/>
       <c r="N182" s="11" t="n"/>
       <c r="O182" s="11" t="n"/>
+      <c r="P182" s="11" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="10" t="n"/>
@@ -22992,6 +23241,7 @@
       <c r="M183" s="11" t="n"/>
       <c r="N183" s="11" t="n"/>
       <c r="O183" s="11" t="n"/>
+      <c r="P183" s="11" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="10" t="n"/>
@@ -23009,6 +23259,7 @@
       <c r="M184" s="11" t="n"/>
       <c r="N184" s="11" t="n"/>
       <c r="O184" s="11" t="n"/>
+      <c r="P184" s="11" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="10" t="n"/>
@@ -23026,6 +23277,7 @@
       <c r="M185" s="11" t="n"/>
       <c r="N185" s="11" t="n"/>
       <c r="O185" s="11" t="n"/>
+      <c r="P185" s="11" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="10" t="n"/>
@@ -23043,6 +23295,7 @@
       <c r="M186" s="11" t="n"/>
       <c r="N186" s="11" t="n"/>
       <c r="O186" s="11" t="n"/>
+      <c r="P186" s="11" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="10" t="n"/>
@@ -23060,6 +23313,7 @@
       <c r="M187" s="11" t="n"/>
       <c r="N187" s="11" t="n"/>
       <c r="O187" s="11" t="n"/>
+      <c r="P187" s="11" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="10" t="n"/>
@@ -23077,6 +23331,7 @@
       <c r="M188" s="11" t="n"/>
       <c r="N188" s="11" t="n"/>
       <c r="O188" s="11" t="n"/>
+      <c r="P188" s="11" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="10" t="n"/>
@@ -23094,6 +23349,7 @@
       <c r="M189" s="11" t="n"/>
       <c r="N189" s="11" t="n"/>
       <c r="O189" s="11" t="n"/>
+      <c r="P189" s="11" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="10" t="n"/>
@@ -23111,6 +23367,7 @@
       <c r="M190" s="11" t="n"/>
       <c r="N190" s="11" t="n"/>
       <c r="O190" s="11" t="n"/>
+      <c r="P190" s="11" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="10" t="n"/>
@@ -23128,6 +23385,7 @@
       <c r="M191" s="11" t="n"/>
       <c r="N191" s="11" t="n"/>
       <c r="O191" s="11" t="n"/>
+      <c r="P191" s="11" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="10" t="n"/>
@@ -23145,6 +23403,7 @@
       <c r="M192" s="11" t="n"/>
       <c r="N192" s="11" t="n"/>
       <c r="O192" s="11" t="n"/>
+      <c r="P192" s="11" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="10" t="n"/>
@@ -23162,6 +23421,7 @@
       <c r="M193" s="11" t="n"/>
       <c r="N193" s="11" t="n"/>
       <c r="O193" s="11" t="n"/>
+      <c r="P193" s="11" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="10" t="n"/>
@@ -23179,6 +23439,7 @@
       <c r="M194" s="11" t="n"/>
       <c r="N194" s="11" t="n"/>
       <c r="O194" s="11" t="n"/>
+      <c r="P194" s="11" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="10" t="n"/>
@@ -23196,6 +23457,7 @@
       <c r="M195" s="11" t="n"/>
       <c r="N195" s="11" t="n"/>
       <c r="O195" s="11" t="n"/>
+      <c r="P195" s="11" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="10" t="n"/>
@@ -23213,6 +23475,7 @@
       <c r="M196" s="11" t="n"/>
       <c r="N196" s="11" t="n"/>
       <c r="O196" s="11" t="n"/>
+      <c r="P196" s="11" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="10" t="n"/>
@@ -23230,6 +23493,7 @@
       <c r="M197" s="11" t="n"/>
       <c r="N197" s="11" t="n"/>
       <c r="O197" s="11" t="n"/>
+      <c r="P197" s="11" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="10" t="n"/>
@@ -23247,6 +23511,7 @@
       <c r="M198" s="11" t="n"/>
       <c r="N198" s="11" t="n"/>
       <c r="O198" s="11" t="n"/>
+      <c r="P198" s="11" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="10" t="n"/>
@@ -23264,6 +23529,7 @@
       <c r="M199" s="11" t="n"/>
       <c r="N199" s="11" t="n"/>
       <c r="O199" s="11" t="n"/>
+      <c r="P199" s="11" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="10" t="n"/>
@@ -23281,6 +23547,7 @@
       <c r="M200" s="11" t="n"/>
       <c r="N200" s="11" t="n"/>
       <c r="O200" s="11" t="n"/>
+      <c r="P200" s="11" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="10" t="n"/>
@@ -23298,6 +23565,7 @@
       <c r="M201" s="11" t="n"/>
       <c r="N201" s="11" t="n"/>
       <c r="O201" s="11" t="n"/>
+      <c r="P201" s="11" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="10" t="n"/>
@@ -23315,6 +23583,7 @@
       <c r="M202" s="11" t="n"/>
       <c r="N202" s="11" t="n"/>
       <c r="O202" s="11" t="n"/>
+      <c r="P202" s="11" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="10" t="n"/>
@@ -23332,6 +23601,7 @@
       <c r="M203" s="11" t="n"/>
       <c r="N203" s="11" t="n"/>
       <c r="O203" s="11" t="n"/>
+      <c r="P203" s="11" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="10" t="n"/>
@@ -23349,6 +23619,7 @@
       <c r="M204" s="11" t="n"/>
       <c r="N204" s="11" t="n"/>
       <c r="O204" s="11" t="n"/>
+      <c r="P204" s="11" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="10" t="n"/>
@@ -23366,6 +23637,7 @@
       <c r="M205" s="11" t="n"/>
       <c r="N205" s="11" t="n"/>
       <c r="O205" s="11" t="n"/>
+      <c r="P205" s="11" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="10" t="n"/>
@@ -23383,6 +23655,7 @@
       <c r="M206" s="11" t="n"/>
       <c r="N206" s="11" t="n"/>
       <c r="O206" s="11" t="n"/>
+      <c r="P206" s="11" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="10" t="n"/>
@@ -23400,6 +23673,7 @@
       <c r="M207" s="11" t="n"/>
       <c r="N207" s="11" t="n"/>
       <c r="O207" s="11" t="n"/>
+      <c r="P207" s="11" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="10" t="n"/>
@@ -23417,6 +23691,7 @@
       <c r="M208" s="11" t="n"/>
       <c r="N208" s="11" t="n"/>
       <c r="O208" s="11" t="n"/>
+      <c r="P208" s="11" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="10" t="n"/>
@@ -23434,6 +23709,7 @@
       <c r="M209" s="11" t="n"/>
       <c r="N209" s="11" t="n"/>
       <c r="O209" s="11" t="n"/>
+      <c r="P209" s="11" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="10" t="n"/>
@@ -23451,6 +23727,7 @@
       <c r="M210" s="11" t="n"/>
       <c r="N210" s="11" t="n"/>
       <c r="O210" s="11" t="n"/>
+      <c r="P210" s="11" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="10" t="n"/>
@@ -23468,6 +23745,7 @@
       <c r="M211" s="11" t="n"/>
       <c r="N211" s="11" t="n"/>
       <c r="O211" s="11" t="n"/>
+      <c r="P211" s="11" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="10" t="n"/>
@@ -23485,6 +23763,7 @@
       <c r="M212" s="11" t="n"/>
       <c r="N212" s="11" t="n"/>
       <c r="O212" s="11" t="n"/>
+      <c r="P212" s="11" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="10" t="n"/>
@@ -23502,6 +23781,7 @@
       <c r="M213" s="11" t="n"/>
       <c r="N213" s="11" t="n"/>
       <c r="O213" s="11" t="n"/>
+      <c r="P213" s="11" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="10" t="n"/>
@@ -23519,6 +23799,7 @@
       <c r="M214" s="11" t="n"/>
       <c r="N214" s="11" t="n"/>
       <c r="O214" s="11" t="n"/>
+      <c r="P214" s="11" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="10" t="n"/>
@@ -23536,6 +23817,7 @@
       <c r="M215" s="11" t="n"/>
       <c r="N215" s="11" t="n"/>
       <c r="O215" s="11" t="n"/>
+      <c r="P215" s="11" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="10" t="n"/>
@@ -23553,6 +23835,7 @@
       <c r="M216" s="11" t="n"/>
       <c r="N216" s="11" t="n"/>
       <c r="O216" s="11" t="n"/>
+      <c r="P216" s="11" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="10" t="n"/>
@@ -23570,6 +23853,7 @@
       <c r="M217" s="11" t="n"/>
       <c r="N217" s="11" t="n"/>
       <c r="O217" s="11" t="n"/>
+      <c r="P217" s="11" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="10" t="n"/>
@@ -23587,6 +23871,7 @@
       <c r="M218" s="11" t="n"/>
       <c r="N218" s="11" t="n"/>
       <c r="O218" s="11" t="n"/>
+      <c r="P218" s="11" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="10" t="n"/>
@@ -23604,6 +23889,7 @@
       <c r="M219" s="11" t="n"/>
       <c r="N219" s="11" t="n"/>
       <c r="O219" s="11" t="n"/>
+      <c r="P219" s="11" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="10" t="n"/>
@@ -23621,6 +23907,7 @@
       <c r="M220" s="11" t="n"/>
       <c r="N220" s="11" t="n"/>
       <c r="O220" s="11" t="n"/>
+      <c r="P220" s="11" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="10" t="n"/>
@@ -23638,6 +23925,7 @@
       <c r="M221" s="11" t="n"/>
       <c r="N221" s="11" t="n"/>
       <c r="O221" s="11" t="n"/>
+      <c r="P221" s="11" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="10" t="n"/>
@@ -23655,6 +23943,7 @@
       <c r="M222" s="11" t="n"/>
       <c r="N222" s="11" t="n"/>
       <c r="O222" s="11" t="n"/>
+      <c r="P222" s="11" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="10" t="n"/>
@@ -23672,6 +23961,7 @@
       <c r="M223" s="11" t="n"/>
       <c r="N223" s="11" t="n"/>
       <c r="O223" s="11" t="n"/>
+      <c r="P223" s="11" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="10" t="n"/>
@@ -23689,6 +23979,7 @@
       <c r="M224" s="11" t="n"/>
       <c r="N224" s="11" t="n"/>
       <c r="O224" s="11" t="n"/>
+      <c r="P224" s="11" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="10" t="n"/>
@@ -23706,6 +23997,7 @@
       <c r="M225" s="11" t="n"/>
       <c r="N225" s="11" t="n"/>
       <c r="O225" s="11" t="n"/>
+      <c r="P225" s="11" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="10" t="n"/>
@@ -23723,6 +24015,7 @@
       <c r="M226" s="11" t="n"/>
       <c r="N226" s="11" t="n"/>
       <c r="O226" s="11" t="n"/>
+      <c r="P226" s="11" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="10" t="n"/>
@@ -23740,6 +24033,7 @@
       <c r="M227" s="11" t="n"/>
       <c r="N227" s="11" t="n"/>
       <c r="O227" s="11" t="n"/>
+      <c r="P227" s="11" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="10" t="n"/>
@@ -23757,6 +24051,7 @@
       <c r="M228" s="11" t="n"/>
       <c r="N228" s="11" t="n"/>
       <c r="O228" s="11" t="n"/>
+      <c r="P228" s="11" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="10" t="n"/>
@@ -23774,6 +24069,7 @@
       <c r="M229" s="11" t="n"/>
       <c r="N229" s="11" t="n"/>
       <c r="O229" s="11" t="n"/>
+      <c r="P229" s="11" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="10" t="n"/>
@@ -23791,6 +24087,7 @@
       <c r="M230" s="11" t="n"/>
       <c r="N230" s="11" t="n"/>
       <c r="O230" s="11" t="n"/>
+      <c r="P230" s="11" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="10" t="n"/>
@@ -23808,6 +24105,7 @@
       <c r="M231" s="11" t="n"/>
       <c r="N231" s="11" t="n"/>
       <c r="O231" s="11" t="n"/>
+      <c r="P231" s="11" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="10" t="n"/>
@@ -23825,6 +24123,7 @@
       <c r="M232" s="11" t="n"/>
       <c r="N232" s="11" t="n"/>
       <c r="O232" s="11" t="n"/>
+      <c r="P232" s="11" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="10" t="n"/>
@@ -23842,6 +24141,7 @@
       <c r="M233" s="11" t="n"/>
       <c r="N233" s="11" t="n"/>
       <c r="O233" s="11" t="n"/>
+      <c r="P233" s="11" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="10" t="n"/>
@@ -23859,6 +24159,7 @@
       <c r="M234" s="11" t="n"/>
       <c r="N234" s="11" t="n"/>
       <c r="O234" s="11" t="n"/>
+      <c r="P234" s="11" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="10" t="n"/>
@@ -23876,6 +24177,7 @@
       <c r="M235" s="11" t="n"/>
       <c r="N235" s="11" t="n"/>
       <c r="O235" s="11" t="n"/>
+      <c r="P235" s="11" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="10" t="n"/>
@@ -23893,6 +24195,7 @@
       <c r="M236" s="11" t="n"/>
       <c r="N236" s="11" t="n"/>
       <c r="O236" s="11" t="n"/>
+      <c r="P236" s="11" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="10" t="n"/>
@@ -23910,6 +24213,7 @@
       <c r="M237" s="11" t="n"/>
       <c r="N237" s="11" t="n"/>
       <c r="O237" s="11" t="n"/>
+      <c r="P237" s="11" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="10" t="n"/>
@@ -23927,6 +24231,7 @@
       <c r="M238" s="11" t="n"/>
       <c r="N238" s="11" t="n"/>
       <c r="O238" s="11" t="n"/>
+      <c r="P238" s="11" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="10" t="n"/>
@@ -23944,6 +24249,7 @@
       <c r="M239" s="11" t="n"/>
       <c r="N239" s="11" t="n"/>
       <c r="O239" s="11" t="n"/>
+      <c r="P239" s="11" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="10" t="n"/>
@@ -23961,6 +24267,7 @@
       <c r="M240" s="11" t="n"/>
       <c r="N240" s="11" t="n"/>
       <c r="O240" s="11" t="n"/>
+      <c r="P240" s="11" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="10" t="n"/>
@@ -23978,6 +24285,7 @@
       <c r="M241" s="11" t="n"/>
       <c r="N241" s="11" t="n"/>
       <c r="O241" s="11" t="n"/>
+      <c r="P241" s="11" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="10" t="n"/>
@@ -23995,6 +24303,7 @@
       <c r="M242" s="11" t="n"/>
       <c r="N242" s="11" t="n"/>
       <c r="O242" s="11" t="n"/>
+      <c r="P242" s="11" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="10" t="n"/>
@@ -24012,6 +24321,7 @@
       <c r="M243" s="11" t="n"/>
       <c r="N243" s="11" t="n"/>
       <c r="O243" s="11" t="n"/>
+      <c r="P243" s="11" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="10" t="n"/>
@@ -24029,6 +24339,7 @@
       <c r="M244" s="11" t="n"/>
       <c r="N244" s="11" t="n"/>
       <c r="O244" s="11" t="n"/>
+      <c r="P244" s="11" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="10" t="n"/>
@@ -24046,6 +24357,7 @@
       <c r="M245" s="11" t="n"/>
       <c r="N245" s="11" t="n"/>
       <c r="O245" s="11" t="n"/>
+      <c r="P245" s="11" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="10" t="n"/>
@@ -24063,6 +24375,7 @@
       <c r="M246" s="11" t="n"/>
       <c r="N246" s="11" t="n"/>
       <c r="O246" s="11" t="n"/>
+      <c r="P246" s="11" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="10" t="n"/>
@@ -24080,6 +24393,7 @@
       <c r="M247" s="11" t="n"/>
       <c r="N247" s="11" t="n"/>
       <c r="O247" s="11" t="n"/>
+      <c r="P247" s="11" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="10" t="n"/>
@@ -24097,6 +24411,7 @@
       <c r="M248" s="11" t="n"/>
       <c r="N248" s="11" t="n"/>
       <c r="O248" s="11" t="n"/>
+      <c r="P248" s="11" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="10" t="n"/>
@@ -24114,6 +24429,7 @@
       <c r="M249" s="11" t="n"/>
       <c r="N249" s="11" t="n"/>
       <c r="O249" s="11" t="n"/>
+      <c r="P249" s="11" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="10" t="n"/>
@@ -24131,6 +24447,7 @@
       <c r="M250" s="11" t="n"/>
       <c r="N250" s="11" t="n"/>
       <c r="O250" s="11" t="n"/>
+      <c r="P250" s="11" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="10" t="n"/>
@@ -24148,6 +24465,7 @@
       <c r="M251" s="11" t="n"/>
       <c r="N251" s="11" t="n"/>
       <c r="O251" s="11" t="n"/>
+      <c r="P251" s="11" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="10" t="n"/>
@@ -24165,6 +24483,7 @@
       <c r="M252" s="11" t="n"/>
       <c r="N252" s="11" t="n"/>
       <c r="O252" s="11" t="n"/>
+      <c r="P252" s="11" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="10" t="n"/>
@@ -24182,6 +24501,7 @@
       <c r="M253" s="11" t="n"/>
       <c r="N253" s="11" t="n"/>
       <c r="O253" s="11" t="n"/>
+      <c r="P253" s="11" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="10" t="n"/>
@@ -24199,6 +24519,7 @@
       <c r="M254" s="11" t="n"/>
       <c r="N254" s="11" t="n"/>
       <c r="O254" s="11" t="n"/>
+      <c r="P254" s="11" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="10" t="n"/>
@@ -24216,6 +24537,7 @@
       <c r="M255" s="11" t="n"/>
       <c r="N255" s="11" t="n"/>
       <c r="O255" s="11" t="n"/>
+      <c r="P255" s="11" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="10" t="n"/>
@@ -24233,6 +24555,7 @@
       <c r="M256" s="11" t="n"/>
       <c r="N256" s="11" t="n"/>
       <c r="O256" s="11" t="n"/>
+      <c r="P256" s="11" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="10" t="n"/>
@@ -24250,6 +24573,7 @@
       <c r="M257" s="11" t="n"/>
       <c r="N257" s="11" t="n"/>
       <c r="O257" s="11" t="n"/>
+      <c r="P257" s="11" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="10" t="n"/>
@@ -24267,6 +24591,7 @@
       <c r="M258" s="11" t="n"/>
       <c r="N258" s="11" t="n"/>
       <c r="O258" s="11" t="n"/>
+      <c r="P258" s="11" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="10" t="n"/>
@@ -24284,6 +24609,7 @@
       <c r="M259" s="11" t="n"/>
       <c r="N259" s="11" t="n"/>
       <c r="O259" s="11" t="n"/>
+      <c r="P259" s="11" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="10" t="n"/>
@@ -24301,6 +24627,7 @@
       <c r="M260" s="11" t="n"/>
       <c r="N260" s="11" t="n"/>
       <c r="O260" s="11" t="n"/>
+      <c r="P260" s="11" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="10" t="n"/>
@@ -24318,6 +24645,7 @@
       <c r="M261" s="11" t="n"/>
       <c r="N261" s="11" t="n"/>
       <c r="O261" s="11" t="n"/>
+      <c r="P261" s="11" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="10" t="n"/>
@@ -24335,6 +24663,7 @@
       <c r="M262" s="11" t="n"/>
       <c r="N262" s="11" t="n"/>
       <c r="O262" s="11" t="n"/>
+      <c r="P262" s="11" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="10" t="n"/>
@@ -24352,6 +24681,7 @@
       <c r="M263" s="11" t="n"/>
       <c r="N263" s="11" t="n"/>
       <c r="O263" s="11" t="n"/>
+      <c r="P263" s="11" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="10" t="n"/>
@@ -24369,6 +24699,7 @@
       <c r="M264" s="11" t="n"/>
       <c r="N264" s="11" t="n"/>
       <c r="O264" s="11" t="n"/>
+      <c r="P264" s="11" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="10" t="n"/>
@@ -24386,6 +24717,7 @@
       <c r="M265" s="11" t="n"/>
       <c r="N265" s="11" t="n"/>
       <c r="O265" s="11" t="n"/>
+      <c r="P265" s="11" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="10" t="n"/>
@@ -24403,6 +24735,7 @@
       <c r="M266" s="11" t="n"/>
       <c r="N266" s="11" t="n"/>
       <c r="O266" s="11" t="n"/>
+      <c r="P266" s="11" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="10" t="n"/>
@@ -24420,6 +24753,7 @@
       <c r="M267" s="11" t="n"/>
       <c r="N267" s="11" t="n"/>
       <c r="O267" s="11" t="n"/>
+      <c r="P267" s="11" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="10" t="n"/>
@@ -24437,6 +24771,7 @@
       <c r="M268" s="11" t="n"/>
       <c r="N268" s="11" t="n"/>
       <c r="O268" s="11" t="n"/>
+      <c r="P268" s="11" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="10" t="n"/>
@@ -24454,6 +24789,7 @@
       <c r="M269" s="11" t="n"/>
       <c r="N269" s="11" t="n"/>
       <c r="O269" s="11" t="n"/>
+      <c r="P269" s="11" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="10" t="n"/>
@@ -24471,6 +24807,7 @@
       <c r="M270" s="11" t="n"/>
       <c r="N270" s="11" t="n"/>
       <c r="O270" s="11" t="n"/>
+      <c r="P270" s="11" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="10" t="n"/>
@@ -24488,6 +24825,7 @@
       <c r="M271" s="11" t="n"/>
       <c r="N271" s="11" t="n"/>
       <c r="O271" s="11" t="n"/>
+      <c r="P271" s="11" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="10" t="n"/>
@@ -24505,6 +24843,7 @@
       <c r="M272" s="11" t="n"/>
       <c r="N272" s="11" t="n"/>
       <c r="O272" s="11" t="n"/>
+      <c r="P272" s="11" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="10" t="n"/>
@@ -24522,6 +24861,7 @@
       <c r="M273" s="11" t="n"/>
       <c r="N273" s="11" t="n"/>
       <c r="O273" s="11" t="n"/>
+      <c r="P273" s="11" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="10" t="n"/>
@@ -24539,6 +24879,7 @@
       <c r="M274" s="11" t="n"/>
       <c r="N274" s="11" t="n"/>
       <c r="O274" s="11" t="n"/>
+      <c r="P274" s="11" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="10" t="n"/>
@@ -24556,6 +24897,7 @@
       <c r="M275" s="11" t="n"/>
       <c r="N275" s="11" t="n"/>
       <c r="O275" s="11" t="n"/>
+      <c r="P275" s="11" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="10" t="n"/>
@@ -24573,6 +24915,7 @@
       <c r="M276" s="11" t="n"/>
       <c r="N276" s="11" t="n"/>
       <c r="O276" s="11" t="n"/>
+      <c r="P276" s="11" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="10" t="n"/>
@@ -24590,6 +24933,7 @@
       <c r="M277" s="11" t="n"/>
       <c r="N277" s="11" t="n"/>
       <c r="O277" s="11" t="n"/>
+      <c r="P277" s="11" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="10" t="n"/>
@@ -24607,6 +24951,7 @@
       <c r="M278" s="11" t="n"/>
       <c r="N278" s="11" t="n"/>
       <c r="O278" s="11" t="n"/>
+      <c r="P278" s="11" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="10" t="n"/>
@@ -24624,6 +24969,7 @@
       <c r="M279" s="11" t="n"/>
       <c r="N279" s="11" t="n"/>
       <c r="O279" s="11" t="n"/>
+      <c r="P279" s="11" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="10" t="n"/>
@@ -24641,6 +24987,7 @@
       <c r="M280" s="11" t="n"/>
       <c r="N280" s="11" t="n"/>
       <c r="O280" s="11" t="n"/>
+      <c r="P280" s="11" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="10" t="n"/>
@@ -24658,6 +25005,7 @@
       <c r="M281" s="11" t="n"/>
       <c r="N281" s="11" t="n"/>
       <c r="O281" s="11" t="n"/>
+      <c r="P281" s="11" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="10" t="n"/>
@@ -24675,6 +25023,7 @@
       <c r="M282" s="11" t="n"/>
       <c r="N282" s="11" t="n"/>
       <c r="O282" s="11" t="n"/>
+      <c r="P282" s="11" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="10" t="n"/>
@@ -24692,6 +25041,7 @@
       <c r="M283" s="11" t="n"/>
       <c r="N283" s="11" t="n"/>
       <c r="O283" s="11" t="n"/>
+      <c r="P283" s="11" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="10" t="n"/>
@@ -24709,6 +25059,7 @@
       <c r="M284" s="11" t="n"/>
       <c r="N284" s="11" t="n"/>
       <c r="O284" s="11" t="n"/>
+      <c r="P284" s="11" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="10" t="n"/>
@@ -24726,6 +25077,7 @@
       <c r="M285" s="11" t="n"/>
       <c r="N285" s="11" t="n"/>
       <c r="O285" s="11" t="n"/>
+      <c r="P285" s="11" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="10" t="n"/>
@@ -24743,6 +25095,7 @@
       <c r="M286" s="11" t="n"/>
       <c r="N286" s="11" t="n"/>
       <c r="O286" s="11" t="n"/>
+      <c r="P286" s="11" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="10" t="n"/>
@@ -24760,6 +25113,7 @@
       <c r="M287" s="11" t="n"/>
       <c r="N287" s="11" t="n"/>
       <c r="O287" s="11" t="n"/>
+      <c r="P287" s="11" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="10" t="n"/>
@@ -24777,6 +25131,7 @@
       <c r="M288" s="11" t="n"/>
       <c r="N288" s="11" t="n"/>
       <c r="O288" s="11" t="n"/>
+      <c r="P288" s="11" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="10" t="n"/>
@@ -24794,6 +25149,7 @@
       <c r="M289" s="11" t="n"/>
       <c r="N289" s="11" t="n"/>
       <c r="O289" s="11" t="n"/>
+      <c r="P289" s="11" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="10" t="n"/>
@@ -24811,6 +25167,7 @@
       <c r="M290" s="11" t="n"/>
       <c r="N290" s="11" t="n"/>
       <c r="O290" s="11" t="n"/>
+      <c r="P290" s="11" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="10" t="n"/>
@@ -24828,6 +25185,7 @@
       <c r="M291" s="11" t="n"/>
       <c r="N291" s="11" t="n"/>
       <c r="O291" s="11" t="n"/>
+      <c r="P291" s="11" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="10" t="n"/>
@@ -24845,6 +25203,7 @@
       <c r="M292" s="11" t="n"/>
       <c r="N292" s="11" t="n"/>
       <c r="O292" s="11" t="n"/>
+      <c r="P292" s="11" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="10" t="n"/>
@@ -24862,6 +25221,7 @@
       <c r="M293" s="11" t="n"/>
       <c r="N293" s="11" t="n"/>
       <c r="O293" s="11" t="n"/>
+      <c r="P293" s="11" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="10" t="n"/>
@@ -24879,6 +25239,7 @@
       <c r="M294" s="11" t="n"/>
       <c r="N294" s="11" t="n"/>
       <c r="O294" s="11" t="n"/>
+      <c r="P294" s="11" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="10" t="n"/>
@@ -24896,6 +25257,7 @@
       <c r="M295" s="11" t="n"/>
       <c r="N295" s="11" t="n"/>
       <c r="O295" s="11" t="n"/>
+      <c r="P295" s="11" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="10" t="n"/>
@@ -24913,6 +25275,7 @@
       <c r="M296" s="11" t="n"/>
       <c r="N296" s="11" t="n"/>
       <c r="O296" s="11" t="n"/>
+      <c r="P296" s="11" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="10" t="n"/>
@@ -24930,6 +25293,7 @@
       <c r="M297" s="11" t="n"/>
       <c r="N297" s="11" t="n"/>
       <c r="O297" s="11" t="n"/>
+      <c r="P297" s="11" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="10" t="n"/>
@@ -24947,6 +25311,7 @@
       <c r="M298" s="11" t="n"/>
       <c r="N298" s="11" t="n"/>
       <c r="O298" s="11" t="n"/>
+      <c r="P298" s="11" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="10" t="n"/>
@@ -24964,6 +25329,7 @@
       <c r="M299" s="11" t="n"/>
       <c r="N299" s="11" t="n"/>
       <c r="O299" s="11" t="n"/>
+      <c r="P299" s="11" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="10" t="n"/>
@@ -24981,6 +25347,7 @@
       <c r="M300" s="11" t="n"/>
       <c r="N300" s="11" t="n"/>
       <c r="O300" s="11" t="n"/>
+      <c r="P300" s="11" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="10" t="n"/>
@@ -24998,6 +25365,7 @@
       <c r="M301" s="11" t="n"/>
       <c r="N301" s="11" t="n"/>
       <c r="O301" s="11" t="n"/>
+      <c r="P301" s="11" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="10" t="n"/>
@@ -25015,6 +25383,7 @@
       <c r="M302" s="11" t="n"/>
       <c r="N302" s="11" t="n"/>
       <c r="O302" s="11" t="n"/>
+      <c r="P302" s="11" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="10" t="n"/>
@@ -25032,6 +25401,7 @@
       <c r="M303" s="11" t="n"/>
       <c r="N303" s="11" t="n"/>
       <c r="O303" s="11" t="n"/>
+      <c r="P303" s="11" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="10" t="n"/>
@@ -25049,6 +25419,7 @@
       <c r="M304" s="11" t="n"/>
       <c r="N304" s="11" t="n"/>
       <c r="O304" s="11" t="n"/>
+      <c r="P304" s="11" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="10" t="n"/>
@@ -25066,6 +25437,7 @@
       <c r="M305" s="11" t="n"/>
       <c r="N305" s="11" t="n"/>
       <c r="O305" s="11" t="n"/>
+      <c r="P305" s="11" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="10" t="n"/>
@@ -25083,12 +25455,13 @@
       <c r="M306" s="11" t="n"/>
       <c r="N306" s="11" t="n"/>
       <c r="O306" s="11" t="n"/>
+      <c r="P306" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A5:P5"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <dataValidations count="14">
     <dataValidation sqref="A6:A306" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revisá el DNI" error="Ingresá solo números, sin puntos ni espacios (por ejemplo 30111222). Si el documento es correcto y tiene otra cantidad de dígitos, aceptá igual." type="custom" errorStyle="warning">

</xml_diff>